<commit_message>
Update Excel files for download functionality
</commit_message>
<xml_diff>
--- a/excel_routes/route_ATZ_RUH_threats.xlsx
+++ b/excel_routes/route_ATZ_RUH_threats.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CODERED\LAB\market_insights\outputs\run_generated_281225_at_07.09\reports\excel_routes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CODERED\LAB\market_insights\outputs\run_generated_311225_at_15.57\reports\excel_routes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D19BCDAA-429F-44E7-B0A6-88EF94F52555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FAB4208-247A-4ADE-9FF1-EE268B07B599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="696" yWindow="3132" windowWidth="15408" windowHeight="7620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="THREAT_ALERT" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="47">
   <si>
     <t>Date</t>
   </si>
@@ -60,16 +60,16 @@
     <t>Currency</t>
   </si>
   <si>
-    <t>28-DEC-25</t>
+    <t>04-JAN-26</t>
   </si>
   <si>
     <t>SM-463</t>
   </si>
   <si>
-    <t>flyadeal F3-612</t>
-  </si>
-  <si>
-    <t>LOW</t>
+    <t>flyadeal F3-606</t>
+  </si>
+  <si>
+    <t>LOW THREAT</t>
   </si>
   <si>
     <t>EGP</t>
@@ -78,75 +78,84 @@
     <t>flyadeal F3-616</t>
   </si>
   <si>
-    <t>flyadeal F3-608</t>
-  </si>
-  <si>
-    <t>flyadeal F3-606</t>
+    <t>Air Arabia Egypt E5-410</t>
+  </si>
+  <si>
+    <t>Air Arabia Egypt E5-415</t>
+  </si>
+  <si>
+    <t>06-JAN-26</t>
+  </si>
+  <si>
+    <t>Nesma Airlines NE-160</t>
+  </si>
+  <si>
+    <t>flynas XY-266</t>
+  </si>
+  <si>
+    <t>EgyptAir MS-649</t>
+  </si>
+  <si>
+    <t>EgyptAir MS-651</t>
+  </si>
+  <si>
+    <t>Saudia SV-320</t>
+  </si>
+  <si>
+    <t>EgyptAir MS-647</t>
+  </si>
+  <si>
+    <t>Saudia SV-324</t>
+  </si>
+  <si>
+    <t>Saudia SV-312</t>
+  </si>
+  <si>
+    <t>Saudia SV-418</t>
+  </si>
+  <si>
+    <t>flynas XY-284</t>
+  </si>
+  <si>
+    <t>07-JAN-26</t>
+  </si>
+  <si>
+    <t>SM-465</t>
+  </si>
+  <si>
+    <t>Nile Air NP-251</t>
+  </si>
+  <si>
+    <t>flynas XY-268</t>
+  </si>
+  <si>
+    <t>flynas XY-264</t>
+  </si>
+  <si>
+    <t>flynas XY-274</t>
+  </si>
+  <si>
+    <t>flynas XY-270</t>
+  </si>
+  <si>
+    <t>flynas XY-276</t>
+  </si>
+  <si>
+    <t>flynas XY-272</t>
+  </si>
+  <si>
+    <t>Saudia SV-310</t>
+  </si>
+  <si>
+    <t>11-JAN-26</t>
+  </si>
+  <si>
+    <t>Nesma Airlines NE-162</t>
   </si>
   <si>
     <t>Nile Air NP-151</t>
   </si>
   <si>
-    <t>flynas XY-266</t>
-  </si>
-  <si>
-    <t>flynas XY-272</t>
-  </si>
-  <si>
-    <t>30-DEC-25</t>
-  </si>
-  <si>
-    <t>Air Arabia Egypt E5-415</t>
-  </si>
-  <si>
-    <t>Nesma Airlines NE-160</t>
-  </si>
-  <si>
-    <t>Air Arabia Egypt E5-410</t>
-  </si>
-  <si>
-    <t>flynas XY-274</t>
-  </si>
-  <si>
-    <t>flynas XY-270</t>
-  </si>
-  <si>
-    <t>Saudia SV-324</t>
-  </si>
-  <si>
-    <t>Saudia SV-312</t>
-  </si>
-  <si>
-    <t>06-JAN-26</t>
-  </si>
-  <si>
-    <t>EgyptAir MS-649</t>
-  </si>
-  <si>
-    <t>EgyptAir MS-651</t>
-  </si>
-  <si>
-    <t>flynas XY-284</t>
-  </si>
-  <si>
-    <t>07-JAN-26</t>
-  </si>
-  <si>
-    <t>SM-465</t>
-  </si>
-  <si>
-    <t>Nile Air NP-251</t>
-  </si>
-  <si>
-    <t>EgyptAir MS-647</t>
-  </si>
-  <si>
-    <t>Saudia SV-310</t>
-  </si>
-  <si>
-    <t>11-JAN-26</t>
-  </si>
-  <si>
     <t>13-JAN-26</t>
   </si>
   <si>
@@ -154,6 +163,9 @@
   </si>
   <si>
     <t>18-JAN-26</t>
+  </si>
+  <si>
+    <t>20-JAN-26</t>
   </si>
 </sst>
 </file>
@@ -541,7 +553,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -552,7 +564,7 @@
     <col min="7" max="7" width="153.44140625" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
     <col min="9" max="9" width="19" customWidth="1"/>
-    <col min="10" max="10" width="8" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
   </cols>
   <sheetData>
@@ -602,13 +614,13 @@
         <v>13</v>
       </c>
       <c r="D2" s="2">
-        <v>5060</v>
+        <v>7340</v>
       </c>
       <c r="E2" s="2">
-        <v>10628</v>
+        <v>12196</v>
       </c>
       <c r="F2" s="2">
-        <v>-5568</v>
+        <v>-4856</v>
       </c>
       <c r="G2" s="2">
         <v>15</v>
@@ -637,13 +649,13 @@
         <v>16</v>
       </c>
       <c r="D3" s="2">
-        <v>5060</v>
+        <v>7340</v>
       </c>
       <c r="E3" s="2">
-        <v>10628</v>
+        <v>12196</v>
       </c>
       <c r="F3" s="2">
-        <v>-5568</v>
+        <v>-4856</v>
       </c>
       <c r="G3" s="2">
         <v>15</v>
@@ -672,22 +684,22 @@
         <v>17</v>
       </c>
       <c r="D4" s="2">
-        <v>5440</v>
+        <v>7564</v>
       </c>
       <c r="E4" s="2">
-        <v>10628</v>
+        <v>12196</v>
       </c>
       <c r="F4" s="2">
-        <v>-5188</v>
+        <v>-4632</v>
       </c>
       <c r="G4" s="2">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H4" s="2">
         <v>30</v>
       </c>
       <c r="I4" s="2">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>14</v>
@@ -707,22 +719,22 @@
         <v>18</v>
       </c>
       <c r="D5" s="2">
-        <v>5440</v>
+        <v>9199</v>
       </c>
       <c r="E5" s="2">
-        <v>10628</v>
+        <v>12196</v>
       </c>
       <c r="F5" s="2">
-        <v>-5188</v>
+        <v>-2997</v>
       </c>
       <c r="G5" s="2">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H5" s="2">
         <v>30</v>
       </c>
       <c r="I5" s="2">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>14</v>
@@ -733,22 +745,22 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D6" s="2">
-        <v>6683</v>
+        <v>5591</v>
       </c>
       <c r="E6" s="2">
-        <v>10628</v>
+        <v>9407</v>
       </c>
       <c r="F6" s="2">
-        <v>-3945</v>
+        <v>-3816</v>
       </c>
       <c r="G6" s="2">
         <v>30</v>
@@ -768,22 +780,22 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D7" s="2">
-        <v>7470</v>
+        <v>5930</v>
       </c>
       <c r="E7" s="2">
-        <v>10628</v>
+        <v>9407</v>
       </c>
       <c r="F7" s="2">
-        <v>-3158</v>
+        <v>-3477</v>
       </c>
       <c r="G7" s="2">
         <v>30</v>
@@ -803,22 +815,22 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D8" s="2">
-        <v>7470</v>
+        <v>6072</v>
       </c>
       <c r="E8" s="2">
-        <v>10628</v>
+        <v>9407</v>
       </c>
       <c r="F8" s="2">
-        <v>-3158</v>
+        <v>-3335</v>
       </c>
       <c r="G8" s="2">
         <v>30</v>
@@ -838,22 +850,22 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D9" s="2">
-        <v>6170</v>
+        <v>6833</v>
       </c>
       <c r="E9" s="2">
-        <v>9423</v>
+        <v>9407</v>
       </c>
       <c r="F9" s="2">
-        <v>-3253</v>
+        <v>-2574</v>
       </c>
       <c r="G9" s="2">
         <v>30</v>
@@ -873,31 +885,31 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>24</v>
-      </c>
       <c r="D10" s="2">
-        <v>6239</v>
+        <v>8101</v>
       </c>
       <c r="E10" s="2">
-        <v>9423</v>
+        <v>9407</v>
       </c>
       <c r="F10" s="2">
-        <v>-3184</v>
+        <v>-1306</v>
       </c>
       <c r="G10" s="2">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="H10" s="2">
         <v>30</v>
       </c>
       <c r="I10" s="2">
-        <v>0</v>
+        <v>-16</v>
       </c>
       <c r="J10" s="3" t="s">
         <v>14</v>
@@ -908,31 +920,31 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D11" s="2">
-        <v>6786</v>
+        <v>8101</v>
       </c>
       <c r="E11" s="2">
-        <v>9423</v>
+        <v>9407</v>
       </c>
       <c r="F11" s="2">
-        <v>-2637</v>
+        <v>-1306</v>
       </c>
       <c r="G11" s="2">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="H11" s="2">
         <v>30</v>
       </c>
       <c r="I11" s="2">
-        <v>0</v>
+        <v>-16</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>14</v>
@@ -943,31 +955,31 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D12" s="2">
-        <v>6836</v>
+        <v>8634</v>
       </c>
       <c r="E12" s="2">
-        <v>9423</v>
+        <v>9407</v>
       </c>
       <c r="F12" s="2">
-        <v>-2587</v>
+        <v>-773</v>
       </c>
       <c r="G12" s="2">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="H12" s="2">
         <v>30</v>
       </c>
       <c r="I12" s="2">
-        <v>0</v>
+        <v>-16</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>14</v>
@@ -978,31 +990,31 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D13" s="2">
-        <v>6836</v>
+        <v>8824</v>
       </c>
       <c r="E13" s="2">
-        <v>9423</v>
+        <v>9407</v>
       </c>
       <c r="F13" s="2">
-        <v>-2587</v>
+        <v>-583</v>
       </c>
       <c r="G13" s="2">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="H13" s="2">
         <v>30</v>
       </c>
       <c r="I13" s="2">
-        <v>0</v>
+        <v>-16</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>14</v>
@@ -1013,31 +1025,31 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D14" s="2">
-        <v>6836</v>
+        <v>9242</v>
       </c>
       <c r="E14" s="2">
-        <v>9423</v>
+        <v>9407</v>
       </c>
       <c r="F14" s="2">
-        <v>-2587</v>
+        <v>-165</v>
       </c>
       <c r="G14" s="2">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="H14" s="2">
         <v>30</v>
       </c>
       <c r="I14" s="2">
-        <v>0</v>
+        <v>-16</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>14</v>
@@ -1048,22 +1060,22 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D15" s="2">
-        <v>9055</v>
+        <v>9242</v>
       </c>
       <c r="E15" s="2">
-        <v>9423</v>
+        <v>9407</v>
       </c>
       <c r="F15" s="2">
-        <v>-368</v>
+        <v>-165</v>
       </c>
       <c r="G15" s="2">
         <v>46</v>
@@ -1083,22 +1095,22 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D16" s="2">
-        <v>9055</v>
+        <v>9242</v>
       </c>
       <c r="E16" s="2">
-        <v>9423</v>
+        <v>9407</v>
       </c>
       <c r="F16" s="2">
-        <v>-368</v>
+        <v>-165</v>
       </c>
       <c r="G16" s="2">
         <v>46</v>
@@ -1118,31 +1130,31 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="D17" s="2">
-        <v>5269</v>
+        <v>9901</v>
       </c>
       <c r="E17" s="2">
-        <v>8624</v>
+        <v>9407</v>
       </c>
       <c r="F17" s="2">
-        <v>-3355</v>
+        <v>494</v>
       </c>
       <c r="G17" s="2">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H17" s="2">
         <v>30</v>
       </c>
       <c r="I17" s="2">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="J17" s="3" t="s">
         <v>14</v>
@@ -1156,19 +1168,19 @@
         <v>30</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D18" s="2">
-        <v>5506</v>
+        <v>5266</v>
       </c>
       <c r="E18" s="2">
-        <v>8624</v>
+        <v>9407</v>
       </c>
       <c r="F18" s="2">
-        <v>-3118</v>
+        <v>-4141</v>
       </c>
       <c r="G18" s="2">
         <v>30</v>
@@ -1191,19 +1203,19 @@
         <v>30</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="D19" s="2">
-        <v>5605</v>
+        <v>6047</v>
       </c>
       <c r="E19" s="2">
-        <v>8624</v>
+        <v>9407</v>
       </c>
       <c r="F19" s="2">
-        <v>-3019</v>
+        <v>-3360</v>
       </c>
       <c r="G19" s="2">
         <v>30</v>
@@ -1226,19 +1238,19 @@
         <v>30</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="D20" s="2">
-        <v>6049</v>
+        <v>6199</v>
       </c>
       <c r="E20" s="2">
-        <v>8624</v>
+        <v>9407</v>
       </c>
       <c r="F20" s="2">
-        <v>-2575</v>
+        <v>-3208</v>
       </c>
       <c r="G20" s="2">
         <v>30</v>
@@ -1261,28 +1273,28 @@
         <v>30</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D21" s="2">
-        <v>7000</v>
+        <v>6199</v>
       </c>
       <c r="E21" s="2">
-        <v>8624</v>
+        <v>9407</v>
       </c>
       <c r="F21" s="2">
-        <v>-1624</v>
+        <v>-3208</v>
       </c>
       <c r="G21" s="2">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="H21" s="2">
         <v>30</v>
       </c>
       <c r="I21" s="2">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>14</v>
@@ -1296,28 +1308,28 @@
         <v>30</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D22" s="2">
-        <v>7558</v>
+        <v>6199</v>
       </c>
       <c r="E22" s="2">
-        <v>8624</v>
+        <v>9407</v>
       </c>
       <c r="F22" s="2">
-        <v>-1066</v>
+        <v>-3208</v>
       </c>
       <c r="G22" s="2">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="H22" s="2">
         <v>30</v>
       </c>
       <c r="I22" s="2">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="J22" s="3" t="s">
         <v>14</v>
@@ -1331,28 +1343,28 @@
         <v>30</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D23" s="2">
-        <v>9905</v>
+        <v>6199</v>
       </c>
       <c r="E23" s="2">
-        <v>8624</v>
+        <v>9407</v>
       </c>
       <c r="F23" s="2">
-        <v>1281</v>
+        <v>-3208</v>
       </c>
       <c r="G23" s="2">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H23" s="2">
         <v>30</v>
       </c>
       <c r="I23" s="2">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="J23" s="3" t="s">
         <v>14</v>
@@ -1363,22 +1375,22 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D24" s="2">
-        <v>5631</v>
+        <v>6833</v>
       </c>
       <c r="E24" s="2">
-        <v>8624</v>
+        <v>9407</v>
       </c>
       <c r="F24" s="2">
-        <v>-2993</v>
+        <v>-2574</v>
       </c>
       <c r="G24" s="2">
         <v>30</v>
@@ -1398,22 +1410,22 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D25" s="2">
-        <v>5631</v>
+        <v>6833</v>
       </c>
       <c r="E25" s="2">
-        <v>8624</v>
+        <v>9407</v>
       </c>
       <c r="F25" s="2">
-        <v>-2993</v>
+        <v>-2574</v>
       </c>
       <c r="G25" s="2">
         <v>30</v>
@@ -1433,22 +1445,22 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="D26" s="2">
-        <v>5743</v>
+        <v>6833</v>
       </c>
       <c r="E26" s="2">
-        <v>8624</v>
+        <v>9407</v>
       </c>
       <c r="F26" s="2">
-        <v>-2881</v>
+        <v>-2574</v>
       </c>
       <c r="G26" s="2">
         <v>30</v>
@@ -1468,22 +1480,22 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="D27" s="2">
-        <v>7000</v>
+        <v>8634</v>
       </c>
       <c r="E27" s="2">
-        <v>8624</v>
+        <v>9407</v>
       </c>
       <c r="F27" s="2">
-        <v>-1624</v>
+        <v>-773</v>
       </c>
       <c r="G27" s="2">
         <v>46</v>
@@ -1503,22 +1515,22 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D28" s="2">
-        <v>7000</v>
+        <v>8634</v>
       </c>
       <c r="E28" s="2">
-        <v>8624</v>
+        <v>9407</v>
       </c>
       <c r="F28" s="2">
-        <v>-1624</v>
+        <v>-773</v>
       </c>
       <c r="G28" s="2">
         <v>46</v>
@@ -1538,22 +1550,22 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="D29" s="2">
-        <v>8117</v>
+        <v>8824</v>
       </c>
       <c r="E29" s="2">
-        <v>8624</v>
+        <v>9407</v>
       </c>
       <c r="F29" s="2">
-        <v>-507</v>
+        <v>-583</v>
       </c>
       <c r="G29" s="2">
         <v>46</v>
@@ -1573,22 +1585,22 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D30" s="2">
-        <v>8434</v>
+        <v>9242</v>
       </c>
       <c r="E30" s="2">
-        <v>8624</v>
+        <v>9407</v>
       </c>
       <c r="F30" s="2">
-        <v>-190</v>
+        <v>-165</v>
       </c>
       <c r="G30" s="2">
         <v>46</v>
@@ -1608,22 +1620,22 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D31" s="2">
-        <v>6480</v>
+        <v>9242</v>
       </c>
       <c r="E31" s="2">
-        <v>7153</v>
+        <v>9407</v>
       </c>
       <c r="F31" s="2">
-        <v>-673</v>
+        <v>-165</v>
       </c>
       <c r="G31" s="2">
         <v>46</v>
@@ -1643,31 +1655,31 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D32" s="2">
-        <v>6582</v>
+        <v>5100</v>
       </c>
       <c r="E32" s="2">
-        <v>7153</v>
+        <v>8608</v>
       </c>
       <c r="F32" s="2">
-        <v>-571</v>
+        <v>-3508</v>
       </c>
       <c r="G32" s="2">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="H32" s="2">
         <v>30</v>
       </c>
       <c r="I32" s="2">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="J32" s="3" t="s">
         <v>14</v>
@@ -1684,25 +1696,25 @@
         <v>12</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D33" s="2">
-        <v>7000</v>
+        <v>5337</v>
       </c>
       <c r="E33" s="2">
-        <v>7812</v>
+        <v>8608</v>
       </c>
       <c r="F33" s="2">
-        <v>-812</v>
+        <v>-3271</v>
       </c>
       <c r="G33" s="2">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="H33" s="2">
         <v>30</v>
       </c>
       <c r="I33" s="2">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="J33" s="3" t="s">
         <v>14</v>
@@ -1719,25 +1731,25 @@
         <v>12</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="D34" s="2">
-        <v>7000</v>
+        <v>5591</v>
       </c>
       <c r="E34" s="2">
-        <v>7812</v>
+        <v>8608</v>
       </c>
       <c r="F34" s="2">
-        <v>-812</v>
+        <v>-3017</v>
       </c>
       <c r="G34" s="2">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="H34" s="2">
         <v>30</v>
       </c>
       <c r="I34" s="2">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="J34" s="3" t="s">
         <v>14</v>
@@ -1754,25 +1766,25 @@
         <v>12</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D35" s="2">
-        <v>7102</v>
+        <v>5629</v>
       </c>
       <c r="E35" s="2">
-        <v>7812</v>
+        <v>8608</v>
       </c>
       <c r="F35" s="2">
-        <v>-710</v>
+        <v>-2979</v>
       </c>
       <c r="G35" s="2">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="H35" s="2">
         <v>30</v>
       </c>
       <c r="I35" s="2">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="J35" s="3" t="s">
         <v>14</v>
@@ -1783,22 +1795,22 @@
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D36" s="2">
-        <v>5605</v>
+        <v>5692</v>
       </c>
       <c r="E36" s="2">
-        <v>8624</v>
+        <v>8608</v>
       </c>
       <c r="F36" s="2">
-        <v>-3019</v>
+        <v>-2916</v>
       </c>
       <c r="G36" s="2">
         <v>30</v>
@@ -1818,22 +1830,22 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="D37" s="2">
-        <v>6049</v>
+        <v>5692</v>
       </c>
       <c r="E37" s="2">
-        <v>8624</v>
+        <v>8608</v>
       </c>
       <c r="F37" s="2">
-        <v>-2575</v>
+        <v>-2916</v>
       </c>
       <c r="G37" s="2">
         <v>30</v>
@@ -1853,31 +1865,31 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D38" s="2">
-        <v>7558</v>
+        <v>5692</v>
       </c>
       <c r="E38" s="2">
-        <v>8624</v>
+        <v>8608</v>
       </c>
       <c r="F38" s="2">
-        <v>-1066</v>
+        <v>-2916</v>
       </c>
       <c r="G38" s="2">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="H38" s="2">
         <v>30</v>
       </c>
       <c r="I38" s="2">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="J38" s="3" t="s">
         <v>14</v>
@@ -1888,31 +1900,31 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C39" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="D39" s="2">
-        <v>8434</v>
+        <v>5692</v>
       </c>
       <c r="E39" s="2">
-        <v>8624</v>
+        <v>8608</v>
       </c>
       <c r="F39" s="2">
-        <v>-190</v>
+        <v>-2916</v>
       </c>
       <c r="G39" s="2">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="H39" s="2">
         <v>30</v>
       </c>
       <c r="I39" s="2">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="J39" s="3" t="s">
         <v>14</v>
@@ -1923,36 +1935,456 @@
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C40" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D40" s="2">
+        <v>5692</v>
+      </c>
+      <c r="E40" s="2">
+        <v>8608</v>
+      </c>
+      <c r="F40" s="2">
+        <v>-2916</v>
+      </c>
+      <c r="G40" s="2">
+        <v>30</v>
+      </c>
+      <c r="H40" s="2">
+        <v>30</v>
+      </c>
+      <c r="I40" s="2">
+        <v>0</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D41" s="2">
+        <v>6985</v>
+      </c>
+      <c r="E41" s="2">
+        <v>8608</v>
+      </c>
+      <c r="F41" s="2">
+        <v>-1623</v>
+      </c>
+      <c r="G41" s="2">
+        <v>46</v>
+      </c>
+      <c r="H41" s="2">
+        <v>30</v>
+      </c>
+      <c r="I41" s="2">
+        <v>-16</v>
+      </c>
+      <c r="J41" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D42" s="2">
+        <v>7087</v>
+      </c>
+      <c r="E42" s="2">
+        <v>8608</v>
+      </c>
+      <c r="F42" s="2">
+        <v>-1521</v>
+      </c>
+      <c r="G42" s="2">
+        <v>46</v>
+      </c>
+      <c r="H42" s="2">
+        <v>30</v>
+      </c>
+      <c r="I42" s="2">
+        <v>-16</v>
+      </c>
+      <c r="J42" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D43" s="2">
+        <v>7911</v>
+      </c>
+      <c r="E43" s="2">
+        <v>8608</v>
+      </c>
+      <c r="F43" s="2">
+        <v>-697</v>
+      </c>
+      <c r="G43" s="2">
+        <v>46</v>
+      </c>
+      <c r="H43" s="2">
+        <v>30</v>
+      </c>
+      <c r="I43" s="2">
+        <v>-16</v>
+      </c>
+      <c r="J43" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D44" s="2">
+        <v>8203</v>
+      </c>
+      <c r="E44" s="2">
+        <v>8608</v>
+      </c>
+      <c r="F44" s="2">
+        <v>-405</v>
+      </c>
+      <c r="G44" s="2">
+        <v>46</v>
+      </c>
+      <c r="H44" s="2">
+        <v>30</v>
+      </c>
+      <c r="I44" s="2">
+        <v>-16</v>
+      </c>
+      <c r="J44" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D45" s="2">
+        <v>4564</v>
+      </c>
+      <c r="E45" s="2">
+        <v>8608</v>
+      </c>
+      <c r="F45" s="2">
+        <v>-4044</v>
+      </c>
+      <c r="G45" s="2">
+        <v>30</v>
+      </c>
+      <c r="H45" s="2">
+        <v>30</v>
+      </c>
+      <c r="I45" s="2">
+        <v>0</v>
+      </c>
+      <c r="J45" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D46" s="2">
+        <v>4792</v>
+      </c>
+      <c r="E46" s="2">
+        <v>8608</v>
+      </c>
+      <c r="F46" s="2">
+        <v>-3816</v>
+      </c>
+      <c r="G46" s="2">
+        <v>30</v>
+      </c>
+      <c r="H46" s="2">
+        <v>30</v>
+      </c>
+      <c r="I46" s="2">
+        <v>0</v>
+      </c>
+      <c r="J46" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D47" s="2">
+        <v>5029</v>
+      </c>
+      <c r="E47" s="2">
+        <v>8608</v>
+      </c>
+      <c r="F47" s="2">
+        <v>-3579</v>
+      </c>
+      <c r="G47" s="2">
+        <v>30</v>
+      </c>
+      <c r="H47" s="2">
+        <v>30</v>
+      </c>
+      <c r="I47" s="2">
+        <v>0</v>
+      </c>
+      <c r="J47" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D48" s="2">
+        <v>8101</v>
+      </c>
+      <c r="E48" s="2">
+        <v>8608</v>
+      </c>
+      <c r="F48" s="2">
+        <v>-507</v>
+      </c>
+      <c r="G48" s="2">
+        <v>46</v>
+      </c>
+      <c r="H48" s="2">
+        <v>30</v>
+      </c>
+      <c r="I48" s="2">
+        <v>-16</v>
+      </c>
+      <c r="J48" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D40" s="2">
-        <v>8117</v>
-      </c>
-      <c r="E40" s="2">
-        <v>8624</v>
-      </c>
-      <c r="F40" s="2">
-        <v>-507</v>
-      </c>
-      <c r="G40" s="2">
+      <c r="C49" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D49" s="2">
+        <v>5029</v>
+      </c>
+      <c r="E49" s="2">
+        <v>8608</v>
+      </c>
+      <c r="F49" s="2">
+        <v>-3579</v>
+      </c>
+      <c r="G49" s="2">
+        <v>30</v>
+      </c>
+      <c r="H49" s="2">
+        <v>30</v>
+      </c>
+      <c r="I49" s="2">
+        <v>0</v>
+      </c>
+      <c r="J49" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D50" s="2">
+        <v>6285</v>
+      </c>
+      <c r="E50" s="2">
+        <v>9407</v>
+      </c>
+      <c r="F50" s="2">
+        <v>-3122</v>
+      </c>
+      <c r="G50" s="2">
+        <v>30</v>
+      </c>
+      <c r="H50" s="2">
+        <v>30</v>
+      </c>
+      <c r="I50" s="2">
+        <v>0</v>
+      </c>
+      <c r="J50" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H40" s="2">
-        <v>30</v>
-      </c>
-      <c r="I40" s="2">
-        <v>-16</v>
-      </c>
-      <c r="J40" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K40" s="2" t="s">
+      <c r="B51" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D51" s="2">
+        <v>5266</v>
+      </c>
+      <c r="E51" s="2">
+        <v>8608</v>
+      </c>
+      <c r="F51" s="2">
+        <v>-3342</v>
+      </c>
+      <c r="G51" s="2">
+        <v>30</v>
+      </c>
+      <c r="H51" s="2">
+        <v>30</v>
+      </c>
+      <c r="I51" s="2">
+        <v>0</v>
+      </c>
+      <c r="J51" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D52" s="2">
+        <v>5266</v>
+      </c>
+      <c r="E52" s="2">
+        <v>8608</v>
+      </c>
+      <c r="F52" s="2">
+        <v>-3342</v>
+      </c>
+      <c r="G52" s="2">
+        <v>30</v>
+      </c>
+      <c r="H52" s="2">
+        <v>30</v>
+      </c>
+      <c r="I52" s="2">
+        <v>0</v>
+      </c>
+      <c r="J52" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K52" s="2" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>